<commit_message>
rework still inprogress, only one test fails
</commit_message>
<xml_diff>
--- a/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/OnExcelIfDateThenDateOk.xlsx
+++ b/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/OnExcelIfDateThenDateOk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/Lexerow/Dev/Lexerow/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="11_2B8C63A238C272CACCFC3B895DC533011B7D74F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{523742F5-23F6-4424-B8C8-F0D0EC2A0C32}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="11_2B8C63A238C272CACCFC3B895DC533011B7D74F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27B7FDBB-72EC-4D1D-8B3D-4EB58F6A4903}"/>
   <bookViews>
-    <workbookView xWindow="4455" yWindow="4470" windowWidth="18900" windowHeight="10515" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11175" yWindow="4290" windowWidth="16155" windowHeight="6975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
     <t>hour</t>
   </si>
   <si>
-    <t>dateTime</t>
+    <t>dateTime, inf!</t>
   </si>
 </sst>
 </file>
@@ -380,7 +380,7 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="16.7109375" customWidth="1"/>
   </cols>

</xml_diff>